<commit_message>
docs(notifications): hoàn thiện tài liệu + quality gate cho Feature 013
Cập nhật CHANGELOG, FEATURE_LOG, GLOSSARY, LESSONS_LEARNED, PROJECT_OVERVIEW,
TASKS, TEST_CASES, openapi.yaml và các guide (admin/user/troubleshooting) để
khớp với hành vi thực tế của tính năng Notifications (bao gồm điều hướng
targetScreen, toast 7 giây, 4 kịch bản click-to-navigate N1-N4).

Thêm ADR 010 (fire-and-forget polling). Cập nhật workflow/STATUS.md và các
file handoff phản ánh quá trình S2/S4/S5 làm lại theo yêu cầu S8 trước khi
ĐẠT quality gate.
</commit_message>
<xml_diff>
--- a/ThiThu_VN_GameDesignDocument.xlsx
+++ b/ThiThu_VN_GameDesignDocument.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/quangnd512/Desktop/claude/quiz_dh/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A95F83E-DD52-1B40-B615-AB0D366076C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B1432C-BD08-2D41-AE34-E1CFD5E2F852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tong quan" sheetId="1" r:id="rId1"/>
@@ -2844,9 +2844,6 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2854,6 +2851,9 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2875,15 +2875,15 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2899,17 +2899,17 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3227,7 +3227,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="83" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="76"/>
@@ -3377,134 +3377,141 @@
       <c r="A17" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="83" t="s">
+      <c r="B17" s="82" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="82"/>
-      <c r="D17" s="82"/>
-      <c r="E17" s="82"/>
-      <c r="F17" s="82"/>
-      <c r="G17" s="82"/>
+      <c r="C17" s="81"/>
+      <c r="D17" s="81"/>
+      <c r="E17" s="81"/>
+      <c r="F17" s="81"/>
+      <c r="G17" s="81"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="80" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="82"/>
-      <c r="D18" s="82"/>
-      <c r="E18" s="82"/>
-      <c r="F18" s="82"/>
-      <c r="G18" s="82"/>
+      <c r="C18" s="81"/>
+      <c r="D18" s="81"/>
+      <c r="E18" s="81"/>
+      <c r="F18" s="81"/>
+      <c r="G18" s="81"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="83" t="s">
+      <c r="B19" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="C19" s="82"/>
-      <c r="D19" s="82"/>
-      <c r="E19" s="82"/>
-      <c r="F19" s="82"/>
-      <c r="G19" s="82"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="81"/>
+      <c r="E19" s="81"/>
+      <c r="F19" s="81"/>
+      <c r="G19" s="81"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="81" t="s">
+      <c r="B20" s="80" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="82"/>
-      <c r="D20" s="82"/>
-      <c r="E20" s="82"/>
-      <c r="F20" s="82"/>
-      <c r="G20" s="82"/>
+      <c r="C20" s="81"/>
+      <c r="D20" s="81"/>
+      <c r="E20" s="81"/>
+      <c r="F20" s="81"/>
+      <c r="G20" s="81"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="83" t="s">
+      <c r="B21" s="82" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="82"/>
-      <c r="D21" s="82"/>
-      <c r="E21" s="82"/>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
+      <c r="E21" s="81"/>
+      <c r="F21" s="81"/>
+      <c r="G21" s="81"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="81" t="s">
+      <c r="B22" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="82"/>
-      <c r="D22" s="82"/>
-      <c r="E22" s="82"/>
-      <c r="F22" s="82"/>
-      <c r="G22" s="82"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="81"/>
+      <c r="F22" s="81"/>
+      <c r="G22" s="81"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="83" t="s">
+      <c r="B23" s="82" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
-      <c r="F23" s="82"/>
-      <c r="G23" s="82"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="81"/>
+      <c r="G23" s="81"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="81" t="s">
+      <c r="B24" s="80" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="82"/>
-      <c r="D24" s="82"/>
-      <c r="E24" s="82"/>
-      <c r="F24" s="82"/>
-      <c r="G24" s="82"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="83" t="s">
+      <c r="B25" s="82" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="82"/>
-      <c r="G25" s="82"/>
+      <c r="C25" s="81"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="81"/>
+      <c r="G25" s="81"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B26" s="81" t="s">
+      <c r="B26" s="80" t="s">
         <v>99</v>
       </c>
-      <c r="C26" s="82"/>
-      <c r="D26" s="82"/>
-      <c r="E26" s="82"/>
-      <c r="F26" s="82"/>
-      <c r="G26" s="82"/>
+      <c r="C26" s="81"/>
+      <c r="D26" s="81"/>
+      <c r="E26" s="81"/>
+      <c r="F26" s="81"/>
+      <c r="G26" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="B18:G18"/>
@@ -3513,13 +3520,6 @@
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4892,7 +4892,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="91" t="s">
         <v>272</v>
       </c>
       <c r="B1" s="76"/>
@@ -5569,7 +5569,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="92" t="s">
+      <c r="A45" s="93" t="s">
         <v>363</v>
       </c>
       <c r="B45" s="76"/>
@@ -5651,7 +5651,7 @@
       <c r="G51" s="76"/>
     </row>
     <row r="52" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="91" t="s">
+      <c r="A52" s="92" t="s">
         <v>374</v>
       </c>
       <c r="B52" s="76"/>
@@ -5662,7 +5662,7 @@
       <c r="G52" s="76"/>
     </row>
     <row r="53" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="91" t="s">
+      <c r="A53" s="92" t="s">
         <v>375</v>
       </c>
       <c r="B53" s="76"/>
@@ -5673,7 +5673,7 @@
       <c r="G53" s="76"/>
     </row>
     <row r="54" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="91" t="s">
+      <c r="A54" s="92" t="s">
         <v>376</v>
       </c>
       <c r="B54" s="76"/>
@@ -5684,7 +5684,7 @@
       <c r="G54" s="76"/>
     </row>
     <row r="55" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="91" t="s">
+      <c r="A55" s="92" t="s">
         <v>377</v>
       </c>
       <c r="B55" s="76"/>
@@ -5695,7 +5695,7 @@
       <c r="G55" s="76"/>
     </row>
     <row r="56" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="91" t="s">
+      <c r="A56" s="92" t="s">
         <v>378</v>
       </c>
       <c r="B56" s="76"/>
@@ -5706,7 +5706,7 @@
       <c r="G56" s="76"/>
     </row>
     <row r="57" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="91" t="s">
+      <c r="A57" s="92" t="s">
         <v>379</v>
       </c>
       <c r="B57" s="76"/>
@@ -5717,7 +5717,7 @@
       <c r="G57" s="76"/>
     </row>
     <row r="58" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="91" t="s">
+      <c r="A58" s="92" t="s">
         <v>380</v>
       </c>
       <c r="B58" s="76"/>
@@ -5728,7 +5728,7 @@
       <c r="G58" s="76"/>
     </row>
     <row r="59" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="91" t="s">
+      <c r="A59" s="92" t="s">
         <v>381</v>
       </c>
       <c r="B59" s="76"/>
@@ -5739,7 +5739,7 @@
       <c r="G59" s="76"/>
     </row>
     <row r="60" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="91" t="s">
+      <c r="A60" s="92" t="s">
         <v>382</v>
       </c>
       <c r="B60" s="76"/>
@@ -5750,7 +5750,7 @@
       <c r="G60" s="76"/>
     </row>
     <row r="61" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="91" t="s">
+      <c r="A61" s="92" t="s">
         <v>383</v>
       </c>
       <c r="B61" s="76"/>
@@ -5762,6 +5762,15 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A54:G54"/>
     <mergeCell ref="A25:G25"/>
@@ -5772,15 +5781,6 @@
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A60:G60"/>
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A58:G58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6665,7 +6665,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="100" t="s">
         <v>501</v>
       </c>
       <c r="B1" s="76"/>
@@ -6697,11 +6697,11 @@
       <c r="A5" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="101" t="s">
         <v>506</v>
       </c>
-      <c r="C5" s="82"/>
-      <c r="D5" s="82"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="81"/>
       <c r="E5" s="57" t="s">
         <v>507</v>
       </c>
@@ -6710,11 +6710,11 @@
       <c r="A6" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="B6" s="99" t="s">
+      <c r="B6" s="102" t="s">
         <v>509</v>
       </c>
-      <c r="C6" s="82"/>
-      <c r="D6" s="82"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="81"/>
       <c r="E6" s="58" t="s">
         <v>510</v>
       </c>
@@ -6723,11 +6723,11 @@
       <c r="A7" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="B7" s="100" t="s">
+      <c r="B7" s="101" t="s">
         <v>512</v>
       </c>
-      <c r="C7" s="82"/>
-      <c r="D7" s="82"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="81"/>
       <c r="E7" s="57" t="s">
         <v>513</v>
       </c>
@@ -6736,11 +6736,11 @@
       <c r="A8" s="4" t="s">
         <v>514</v>
       </c>
-      <c r="B8" s="99" t="s">
+      <c r="B8" s="102" t="s">
         <v>515</v>
       </c>
-      <c r="C8" s="82"/>
-      <c r="D8" s="82"/>
+      <c r="C8" s="81"/>
+      <c r="D8" s="81"/>
       <c r="E8" s="58" t="s">
         <v>516</v>
       </c>
@@ -6749,11 +6749,11 @@
       <c r="A9" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="B9" s="100" t="s">
+      <c r="B9" s="101" t="s">
         <v>518</v>
       </c>
-      <c r="C9" s="82"/>
-      <c r="D9" s="82"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="81"/>
       <c r="E9" s="57" t="s">
         <v>510</v>
       </c>
@@ -6782,11 +6782,11 @@
       <c r="A13" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="B13" s="100" t="s">
+      <c r="B13" s="101" t="s">
         <v>521</v>
       </c>
-      <c r="C13" s="82"/>
-      <c r="D13" s="82"/>
+      <c r="C13" s="81"/>
+      <c r="D13" s="81"/>
       <c r="E13" s="57" t="s">
         <v>522</v>
       </c>
@@ -6795,11 +6795,11 @@
       <c r="A14" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="B14" s="99" t="s">
+      <c r="B14" s="102" t="s">
         <v>524</v>
       </c>
-      <c r="C14" s="82"/>
-      <c r="D14" s="82"/>
+      <c r="C14" s="81"/>
+      <c r="D14" s="81"/>
       <c r="E14" s="58" t="s">
         <v>525</v>
       </c>
@@ -6808,11 +6808,11 @@
       <c r="A15" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B15" s="100" t="s">
+      <c r="B15" s="101" t="s">
         <v>527</v>
       </c>
-      <c r="C15" s="82"/>
-      <c r="D15" s="82"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
       <c r="E15" s="57" t="s">
         <v>528</v>
       </c>
@@ -6821,11 +6821,11 @@
       <c r="A16" s="4" t="s">
         <v>529</v>
       </c>
-      <c r="B16" s="99" t="s">
+      <c r="B16" s="102" t="s">
         <v>530</v>
       </c>
-      <c r="C16" s="82"/>
-      <c r="D16" s="82"/>
+      <c r="C16" s="81"/>
+      <c r="D16" s="81"/>
       <c r="E16" s="58" t="s">
         <v>531</v>
       </c>
@@ -6834,11 +6834,11 @@
       <c r="A17" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="B17" s="100" t="s">
+      <c r="B17" s="101" t="s">
         <v>533</v>
       </c>
-      <c r="C17" s="82"/>
-      <c r="D17" s="82"/>
+      <c r="C17" s="81"/>
+      <c r="D17" s="81"/>
       <c r="E17" s="57" t="s">
         <v>534</v>
       </c>
@@ -6867,11 +6867,11 @@
       <c r="A21" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="B21" s="100" t="s">
+      <c r="B21" s="101" t="s">
         <v>537</v>
       </c>
-      <c r="C21" s="82"/>
-      <c r="D21" s="82"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
       <c r="E21" s="57" t="s">
         <v>538</v>
       </c>
@@ -6880,11 +6880,11 @@
       <c r="A22" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="B22" s="99" t="s">
+      <c r="B22" s="102" t="s">
         <v>540</v>
       </c>
-      <c r="C22" s="82"/>
-      <c r="D22" s="82"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
       <c r="E22" s="58" t="s">
         <v>541</v>
       </c>
@@ -6893,11 +6893,11 @@
       <c r="A23" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B23" s="100" t="s">
+      <c r="B23" s="101" t="s">
         <v>543</v>
       </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
       <c r="E23" s="57" t="s">
         <v>544</v>
       </c>
@@ -6906,11 +6906,11 @@
       <c r="A24" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="B24" s="99" t="s">
+      <c r="B24" s="102" t="s">
         <v>546</v>
       </c>
-      <c r="C24" s="82"/>
-      <c r="D24" s="82"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
       <c r="E24" s="58" t="s">
         <v>547</v>
       </c>
@@ -6942,11 +6942,11 @@
       <c r="B29" s="11" t="s">
         <v>553</v>
       </c>
-      <c r="C29" s="101" t="s">
+      <c r="C29" s="99" t="s">
         <v>554</v>
       </c>
-      <c r="D29" s="82"/>
-      <c r="E29" s="82"/>
+      <c r="D29" s="81"/>
+      <c r="E29" s="81"/>
     </row>
     <row r="30" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
@@ -6955,11 +6955,11 @@
       <c r="B30" s="16" t="s">
         <v>556</v>
       </c>
-      <c r="C30" s="81" t="s">
+      <c r="C30" s="80" t="s">
         <v>557</v>
       </c>
-      <c r="D30" s="82"/>
-      <c r="E30" s="82"/>
+      <c r="D30" s="81"/>
+      <c r="E30" s="81"/>
     </row>
     <row r="31" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
@@ -6968,11 +6968,11 @@
       <c r="B31" s="11" t="s">
         <v>559</v>
       </c>
-      <c r="C31" s="101" t="s">
+      <c r="C31" s="99" t="s">
         <v>560</v>
       </c>
-      <c r="D31" s="82"/>
-      <c r="E31" s="82"/>
+      <c r="D31" s="81"/>
+      <c r="E31" s="81"/>
     </row>
     <row r="32" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
@@ -6981,11 +6981,11 @@
       <c r="B32" s="16" t="s">
         <v>562</v>
       </c>
-      <c r="C32" s="81" t="s">
+      <c r="C32" s="80" t="s">
         <v>563</v>
       </c>
-      <c r="D32" s="82"/>
-      <c r="E32" s="82"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="81"/>
     </row>
     <row r="33" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
@@ -6994,11 +6994,11 @@
       <c r="B33" s="11" t="s">
         <v>565</v>
       </c>
-      <c r="C33" s="101" t="s">
+      <c r="C33" s="99" t="s">
         <v>566</v>
       </c>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
+      <c r="D33" s="81"/>
+      <c r="E33" s="81"/>
     </row>
     <row r="34" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
@@ -7007,11 +7007,11 @@
       <c r="B34" s="16" t="s">
         <v>568</v>
       </c>
-      <c r="C34" s="81" t="s">
+      <c r="C34" s="80" t="s">
         <v>569</v>
       </c>
-      <c r="D34" s="82"/>
-      <c r="E34" s="82"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="81"/>
     </row>
     <row r="35" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
@@ -7020,11 +7020,11 @@
       <c r="B35" s="11" t="s">
         <v>571</v>
       </c>
-      <c r="C35" s="101" t="s">
+      <c r="C35" s="99" t="s">
         <v>572</v>
       </c>
-      <c r="D35" s="82"/>
-      <c r="E35" s="82"/>
+      <c r="D35" s="81"/>
+      <c r="E35" s="81"/>
     </row>
     <row r="36" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
@@ -7033,14 +7033,25 @@
       <c r="B36" s="16" t="s">
         <v>574</v>
       </c>
-      <c r="C36" s="81" t="s">
+      <c r="C36" s="80" t="s">
         <v>575</v>
       </c>
-      <c r="D36" s="82"/>
-      <c r="E36" s="82"/>
+      <c r="D36" s="81"/>
+      <c r="E36" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="C35:E35"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C36:E36"/>
@@ -7057,17 +7068,6 @@
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="C29:E29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7326,78 +7326,78 @@
       <c r="A21" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="B21" s="100" t="s">
+      <c r="B21" s="101" t="s">
         <v>636</v>
       </c>
-      <c r="C21" s="82"/>
-      <c r="D21" s="82"/>
-      <c r="E21" s="82"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
+      <c r="E21" s="81"/>
     </row>
     <row r="22" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>637</v>
       </c>
-      <c r="B22" s="99" t="s">
+      <c r="B22" s="102" t="s">
         <v>638</v>
       </c>
-      <c r="C22" s="82"/>
-      <c r="D22" s="82"/>
-      <c r="E22" s="82"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="81"/>
     </row>
     <row r="23" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="B23" s="100" t="s">
+      <c r="B23" s="101" t="s">
         <v>640</v>
       </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="81"/>
     </row>
     <row r="24" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>641</v>
       </c>
-      <c r="B24" s="99" t="s">
+      <c r="B24" s="102" t="s">
         <v>642</v>
       </c>
-      <c r="C24" s="82"/>
-      <c r="D24" s="82"/>
-      <c r="E24" s="82"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
     </row>
     <row r="25" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="B25" s="100" t="s">
+      <c r="B25" s="101" t="s">
         <v>644</v>
       </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
+      <c r="C25" s="81"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="81"/>
     </row>
     <row r="26" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>645</v>
       </c>
-      <c r="B26" s="99" t="s">
+      <c r="B26" s="102" t="s">
         <v>646</v>
       </c>
-      <c r="C26" s="82"/>
-      <c r="D26" s="82"/>
-      <c r="E26" s="82"/>
+      <c r="C26" s="81"/>
+      <c r="D26" s="81"/>
+      <c r="E26" s="81"/>
     </row>
     <row r="27" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="B27" s="100" t="s">
+      <c r="B27" s="101" t="s">
         <v>648</v>
       </c>
-      <c r="C27" s="82"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="82"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="81"/>
+      <c r="E27" s="81"/>
     </row>
     <row r="29" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="89" t="s">
@@ -7412,78 +7412,78 @@
       <c r="A30" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="B30" s="100" t="s">
+      <c r="B30" s="101" t="s">
         <v>651</v>
       </c>
-      <c r="C30" s="82"/>
-      <c r="D30" s="82"/>
-      <c r="E30" s="82"/>
+      <c r="C30" s="81"/>
+      <c r="D30" s="81"/>
+      <c r="E30" s="81"/>
     </row>
     <row r="31" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="B31" s="99" t="s">
+      <c r="B31" s="102" t="s">
         <v>653</v>
       </c>
-      <c r="C31" s="82"/>
-      <c r="D31" s="82"/>
-      <c r="E31" s="82"/>
+      <c r="C31" s="81"/>
+      <c r="D31" s="81"/>
+      <c r="E31" s="81"/>
     </row>
     <row r="32" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="B32" s="100" t="s">
+      <c r="B32" s="101" t="s">
         <v>655</v>
       </c>
-      <c r="C32" s="82"/>
-      <c r="D32" s="82"/>
-      <c r="E32" s="82"/>
+      <c r="C32" s="81"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="81"/>
     </row>
     <row r="33" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>656</v>
       </c>
-      <c r="B33" s="99" t="s">
+      <c r="B33" s="102" t="s">
         <v>657</v>
       </c>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
+      <c r="C33" s="81"/>
+      <c r="D33" s="81"/>
+      <c r="E33" s="81"/>
     </row>
     <row r="34" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="B34" s="100" t="s">
+      <c r="B34" s="101" t="s">
         <v>658</v>
       </c>
-      <c r="C34" s="82"/>
-      <c r="D34" s="82"/>
-      <c r="E34" s="82"/>
+      <c r="C34" s="81"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="81"/>
     </row>
     <row r="35" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="B35" s="99" t="s">
+      <c r="B35" s="102" t="s">
         <v>660</v>
       </c>
-      <c r="C35" s="82"/>
-      <c r="D35" s="82"/>
-      <c r="E35" s="82"/>
+      <c r="C35" s="81"/>
+      <c r="D35" s="81"/>
+      <c r="E35" s="81"/>
     </row>
     <row r="36" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="B36" s="100" t="s">
+      <c r="B36" s="101" t="s">
         <v>662</v>
       </c>
-      <c r="C36" s="82"/>
-      <c r="D36" s="82"/>
-      <c r="E36" s="82"/>
+      <c r="C36" s="81"/>
+      <c r="D36" s="81"/>
+      <c r="E36" s="81"/>
     </row>
     <row r="38" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="87" t="s">
@@ -7498,103 +7498,115 @@
       <c r="A39" s="2" t="s">
         <v>664</v>
       </c>
-      <c r="B39" s="100" t="s">
+      <c r="B39" s="101" t="s">
         <v>665</v>
       </c>
-      <c r="C39" s="82"/>
-      <c r="D39" s="82"/>
-      <c r="E39" s="82"/>
+      <c r="C39" s="81"/>
+      <c r="D39" s="81"/>
+      <c r="E39" s="81"/>
     </row>
     <row r="40" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>666</v>
       </c>
-      <c r="B40" s="99" t="s">
+      <c r="B40" s="102" t="s">
         <v>667</v>
       </c>
-      <c r="C40" s="82"/>
-      <c r="D40" s="82"/>
-      <c r="E40" s="82"/>
+      <c r="C40" s="81"/>
+      <c r="D40" s="81"/>
+      <c r="E40" s="81"/>
     </row>
     <row r="41" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="B41" s="100" t="s">
+      <c r="B41" s="101" t="s">
         <v>668</v>
       </c>
-      <c r="C41" s="82"/>
-      <c r="D41" s="82"/>
-      <c r="E41" s="82"/>
+      <c r="C41" s="81"/>
+      <c r="D41" s="81"/>
+      <c r="E41" s="81"/>
     </row>
     <row r="42" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>669</v>
       </c>
-      <c r="B42" s="99" t="s">
+      <c r="B42" s="102" t="s">
         <v>670</v>
       </c>
-      <c r="C42" s="82"/>
-      <c r="D42" s="82"/>
-      <c r="E42" s="82"/>
+      <c r="C42" s="81"/>
+      <c r="D42" s="81"/>
+      <c r="E42" s="81"/>
     </row>
     <row r="43" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="B43" s="100" t="s">
+      <c r="B43" s="101" t="s">
         <v>672</v>
       </c>
-      <c r="C43" s="82"/>
-      <c r="D43" s="82"/>
-      <c r="E43" s="82"/>
+      <c r="C43" s="81"/>
+      <c r="D43" s="81"/>
+      <c r="E43" s="81"/>
     </row>
     <row r="44" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>673</v>
       </c>
-      <c r="B44" s="99" t="s">
+      <c r="B44" s="102" t="s">
         <v>674</v>
       </c>
-      <c r="C44" s="82"/>
-      <c r="D44" s="82"/>
-      <c r="E44" s="82"/>
+      <c r="C44" s="81"/>
+      <c r="D44" s="81"/>
+      <c r="E44" s="81"/>
     </row>
     <row r="45" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="B45" s="100" t="s">
+      <c r="B45" s="101" t="s">
         <v>676</v>
       </c>
-      <c r="C45" s="82"/>
-      <c r="D45" s="82"/>
-      <c r="E45" s="82"/>
+      <c r="C45" s="81"/>
+      <c r="D45" s="81"/>
+      <c r="E45" s="81"/>
     </row>
     <row r="46" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>677</v>
       </c>
-      <c r="B46" s="99" t="s">
+      <c r="B46" s="102" t="s">
         <v>678</v>
       </c>
-      <c r="C46" s="82"/>
-      <c r="D46" s="82"/>
-      <c r="E46" s="82"/>
+      <c r="C46" s="81"/>
+      <c r="D46" s="81"/>
+      <c r="E46" s="81"/>
     </row>
     <row r="47" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>679</v>
       </c>
-      <c r="B47" s="100" t="s">
+      <c r="B47" s="101" t="s">
         <v>680</v>
       </c>
-      <c r="C47" s="82"/>
-      <c r="D47" s="82"/>
-      <c r="E47" s="82"/>
+      <c r="C47" s="81"/>
+      <c r="D47" s="81"/>
+      <c r="E47" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B33:E33"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="B22:E22"/>
@@ -7611,18 +7623,6 @@
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="B34:E34"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B33:E33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mobile): add mobile foundation (auth, navigation, config, storage)
- Auth: Google Sign-In, Apple Sign-In, Firebase integration
- Navigation: root navigator, stack/tab structure, type-safe routing
- Config: environment setup, theme, subject constants
- Storage: secure token storage via expo-secure-store
- UI: primary button, network banner, splash screen
- Docs: API spec, user guide, test cases, code review log
- DevOps: EAS build config, GitHub CI/security workflows, git hooks

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ThiThu_VN_GameDesignDocument.xlsx
+++ b/ThiThu_VN_GameDesignDocument.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/quangnd512/Desktop/claude/quiz_dh/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B1432C-BD08-2D41-AE34-E1CFD5E2F852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A552429D-920D-1044-9795-91889B89AF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +25,7 @@
     <sheet name="Prompts AI" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2844,6 +2845,9 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2851,9 +2855,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2875,16 +2876,16 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2899,17 +2900,17 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3227,7 +3228,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="80" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="76"/>
@@ -3377,141 +3378,134 @@
       <c r="A17" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="82" t="s">
+      <c r="B17" s="83" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="81"/>
-      <c r="D17" s="81"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="81"/>
-      <c r="G17" s="81"/>
+      <c r="C17" s="82"/>
+      <c r="D17" s="82"/>
+      <c r="E17" s="82"/>
+      <c r="F17" s="82"/>
+      <c r="G17" s="82"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="80" t="s">
+      <c r="B18" s="81" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="81"/>
-      <c r="D18" s="81"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="81"/>
-      <c r="G18" s="81"/>
+      <c r="C18" s="82"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="82"/>
+      <c r="F18" s="82"/>
+      <c r="G18" s="82"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="82" t="s">
+      <c r="B19" s="83" t="s">
         <v>85</v>
       </c>
-      <c r="C19" s="81"/>
-      <c r="D19" s="81"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="81"/>
-      <c r="G19" s="81"/>
+      <c r="C19" s="82"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="82"/>
+      <c r="G19" s="82"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="80" t="s">
+      <c r="B20" s="81" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="81"/>
-      <c r="D20" s="81"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="81"/>
-      <c r="G20" s="81"/>
+      <c r="C20" s="82"/>
+      <c r="D20" s="82"/>
+      <c r="E20" s="82"/>
+      <c r="F20" s="82"/>
+      <c r="G20" s="82"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="82" t="s">
+      <c r="B21" s="83" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="81"/>
-      <c r="G21" s="81"/>
+      <c r="C21" s="82"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="82"/>
+      <c r="G21" s="82"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="80" t="s">
+      <c r="B22" s="81" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="81"/>
-      <c r="D22" s="81"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="81"/>
-      <c r="G22" s="81"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="82"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="82"/>
+      <c r="G22" s="82"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="82" t="s">
+      <c r="B23" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="81"/>
-      <c r="D23" s="81"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="81"/>
-      <c r="G23" s="81"/>
+      <c r="C23" s="82"/>
+      <c r="D23" s="82"/>
+      <c r="E23" s="82"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="82"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="80" t="s">
+      <c r="B24" s="81" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="81"/>
-      <c r="D24" s="81"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="81"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="82" t="s">
+      <c r="B25" s="83" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="81"/>
-      <c r="D25" s="81"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="81"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="82"/>
+      <c r="E25" s="82"/>
+      <c r="F25" s="82"/>
+      <c r="G25" s="82"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B26" s="80" t="s">
+      <c r="B26" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="C26" s="81"/>
-      <c r="D26" s="81"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="81"/>
+      <c r="C26" s="82"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="82"/>
+      <c r="F26" s="82"/>
+      <c r="G26" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="B18:G18"/>
@@ -3520,6 +3514,13 @@
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4892,7 +4893,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="93" t="s">
         <v>272</v>
       </c>
       <c r="B1" s="76"/>
@@ -5569,7 +5570,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="93" t="s">
+      <c r="A45" s="92" t="s">
         <v>363</v>
       </c>
       <c r="B45" s="76"/>
@@ -5651,7 +5652,7 @@
       <c r="G51" s="76"/>
     </row>
     <row r="52" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="92" t="s">
+      <c r="A52" s="91" t="s">
         <v>374</v>
       </c>
       <c r="B52" s="76"/>
@@ -5662,7 +5663,7 @@
       <c r="G52" s="76"/>
     </row>
     <row r="53" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="92" t="s">
+      <c r="A53" s="91" t="s">
         <v>375</v>
       </c>
       <c r="B53" s="76"/>
@@ -5673,7 +5674,7 @@
       <c r="G53" s="76"/>
     </row>
     <row r="54" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="92" t="s">
+      <c r="A54" s="91" t="s">
         <v>376</v>
       </c>
       <c r="B54" s="76"/>
@@ -5684,7 +5685,7 @@
       <c r="G54" s="76"/>
     </row>
     <row r="55" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="92" t="s">
+      <c r="A55" s="91" t="s">
         <v>377</v>
       </c>
       <c r="B55" s="76"/>
@@ -5695,7 +5696,7 @@
       <c r="G55" s="76"/>
     </row>
     <row r="56" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="92" t="s">
+      <c r="A56" s="91" t="s">
         <v>378</v>
       </c>
       <c r="B56" s="76"/>
@@ -5706,7 +5707,7 @@
       <c r="G56" s="76"/>
     </row>
     <row r="57" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="92" t="s">
+      <c r="A57" s="91" t="s">
         <v>379</v>
       </c>
       <c r="B57" s="76"/>
@@ -5717,7 +5718,7 @@
       <c r="G57" s="76"/>
     </row>
     <row r="58" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="92" t="s">
+      <c r="A58" s="91" t="s">
         <v>380</v>
       </c>
       <c r="B58" s="76"/>
@@ -5728,7 +5729,7 @@
       <c r="G58" s="76"/>
     </row>
     <row r="59" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="92" t="s">
+      <c r="A59" s="91" t="s">
         <v>381</v>
       </c>
       <c r="B59" s="76"/>
@@ -5739,7 +5740,7 @@
       <c r="G59" s="76"/>
     </row>
     <row r="60" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="92" t="s">
+      <c r="A60" s="91" t="s">
         <v>382</v>
       </c>
       <c r="B60" s="76"/>
@@ -5750,7 +5751,7 @@
       <c r="G60" s="76"/>
     </row>
     <row r="61" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="92" t="s">
+      <c r="A61" s="91" t="s">
         <v>383</v>
       </c>
       <c r="B61" s="76"/>
@@ -5762,15 +5763,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A60:G60"/>
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A54:G54"/>
     <mergeCell ref="A25:G25"/>
@@ -5781,6 +5773,15 @@
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A58:G58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6665,7 +6666,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="102" t="s">
         <v>501</v>
       </c>
       <c r="B1" s="76"/>
@@ -6697,11 +6698,11 @@
       <c r="A5" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="B5" s="101" t="s">
+      <c r="B5" s="100" t="s">
         <v>506</v>
       </c>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
       <c r="E5" s="57" t="s">
         <v>507</v>
       </c>
@@ -6710,11 +6711,11 @@
       <c r="A6" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="B6" s="102" t="s">
+      <c r="B6" s="99" t="s">
         <v>509</v>
       </c>
-      <c r="C6" s="81"/>
-      <c r="D6" s="81"/>
+      <c r="C6" s="82"/>
+      <c r="D6" s="82"/>
       <c r="E6" s="58" t="s">
         <v>510</v>
       </c>
@@ -6723,11 +6724,11 @@
       <c r="A7" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="B7" s="101" t="s">
+      <c r="B7" s="100" t="s">
         <v>512</v>
       </c>
-      <c r="C7" s="81"/>
-      <c r="D7" s="81"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
       <c r="E7" s="57" t="s">
         <v>513</v>
       </c>
@@ -6736,11 +6737,11 @@
       <c r="A8" s="4" t="s">
         <v>514</v>
       </c>
-      <c r="B8" s="102" t="s">
+      <c r="B8" s="99" t="s">
         <v>515</v>
       </c>
-      <c r="C8" s="81"/>
-      <c r="D8" s="81"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
       <c r="E8" s="58" t="s">
         <v>516</v>
       </c>
@@ -6749,11 +6750,11 @@
       <c r="A9" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="B9" s="101" t="s">
+      <c r="B9" s="100" t="s">
         <v>518</v>
       </c>
-      <c r="C9" s="81"/>
-      <c r="D9" s="81"/>
+      <c r="C9" s="82"/>
+      <c r="D9" s="82"/>
       <c r="E9" s="57" t="s">
         <v>510</v>
       </c>
@@ -6782,11 +6783,11 @@
       <c r="A13" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="B13" s="101" t="s">
+      <c r="B13" s="100" t="s">
         <v>521</v>
       </c>
-      <c r="C13" s="81"/>
-      <c r="D13" s="81"/>
+      <c r="C13" s="82"/>
+      <c r="D13" s="82"/>
       <c r="E13" s="57" t="s">
         <v>522</v>
       </c>
@@ -6795,11 +6796,11 @@
       <c r="A14" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="B14" s="102" t="s">
+      <c r="B14" s="99" t="s">
         <v>524</v>
       </c>
-      <c r="C14" s="81"/>
-      <c r="D14" s="81"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
       <c r="E14" s="58" t="s">
         <v>525</v>
       </c>
@@ -6808,11 +6809,11 @@
       <c r="A15" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B15" s="101" t="s">
+      <c r="B15" s="100" t="s">
         <v>527</v>
       </c>
-      <c r="C15" s="81"/>
-      <c r="D15" s="81"/>
+      <c r="C15" s="82"/>
+      <c r="D15" s="82"/>
       <c r="E15" s="57" t="s">
         <v>528</v>
       </c>
@@ -6821,11 +6822,11 @@
       <c r="A16" s="4" t="s">
         <v>529</v>
       </c>
-      <c r="B16" s="102" t="s">
+      <c r="B16" s="99" t="s">
         <v>530</v>
       </c>
-      <c r="C16" s="81"/>
-      <c r="D16" s="81"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
       <c r="E16" s="58" t="s">
         <v>531</v>
       </c>
@@ -6834,11 +6835,11 @@
       <c r="A17" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="B17" s="101" t="s">
+      <c r="B17" s="100" t="s">
         <v>533</v>
       </c>
-      <c r="C17" s="81"/>
-      <c r="D17" s="81"/>
+      <c r="C17" s="82"/>
+      <c r="D17" s="82"/>
       <c r="E17" s="57" t="s">
         <v>534</v>
       </c>
@@ -6867,11 +6868,11 @@
       <c r="A21" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="B21" s="101" t="s">
+      <c r="B21" s="100" t="s">
         <v>537</v>
       </c>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
+      <c r="C21" s="82"/>
+      <c r="D21" s="82"/>
       <c r="E21" s="57" t="s">
         <v>538</v>
       </c>
@@ -6880,11 +6881,11 @@
       <c r="A22" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="B22" s="102" t="s">
+      <c r="B22" s="99" t="s">
         <v>540</v>
       </c>
-      <c r="C22" s="81"/>
-      <c r="D22" s="81"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="82"/>
       <c r="E22" s="58" t="s">
         <v>541</v>
       </c>
@@ -6893,11 +6894,11 @@
       <c r="A23" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B23" s="101" t="s">
+      <c r="B23" s="100" t="s">
         <v>543</v>
       </c>
-      <c r="C23" s="81"/>
-      <c r="D23" s="81"/>
+      <c r="C23" s="82"/>
+      <c r="D23" s="82"/>
       <c r="E23" s="57" t="s">
         <v>544</v>
       </c>
@@ -6906,11 +6907,11 @@
       <c r="A24" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="B24" s="102" t="s">
+      <c r="B24" s="99" t="s">
         <v>546</v>
       </c>
-      <c r="C24" s="81"/>
-      <c r="D24" s="81"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
       <c r="E24" s="58" t="s">
         <v>547</v>
       </c>
@@ -6942,11 +6943,11 @@
       <c r="B29" s="11" t="s">
         <v>553</v>
       </c>
-      <c r="C29" s="99" t="s">
+      <c r="C29" s="101" t="s">
         <v>554</v>
       </c>
-      <c r="D29" s="81"/>
-      <c r="E29" s="81"/>
+      <c r="D29" s="82"/>
+      <c r="E29" s="82"/>
     </row>
     <row r="30" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
@@ -6955,11 +6956,11 @@
       <c r="B30" s="16" t="s">
         <v>556</v>
       </c>
-      <c r="C30" s="80" t="s">
+      <c r="C30" s="81" t="s">
         <v>557</v>
       </c>
-      <c r="D30" s="81"/>
-      <c r="E30" s="81"/>
+      <c r="D30" s="82"/>
+      <c r="E30" s="82"/>
     </row>
     <row r="31" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
@@ -6968,11 +6969,11 @@
       <c r="B31" s="11" t="s">
         <v>559</v>
       </c>
-      <c r="C31" s="99" t="s">
+      <c r="C31" s="101" t="s">
         <v>560</v>
       </c>
-      <c r="D31" s="81"/>
-      <c r="E31" s="81"/>
+      <c r="D31" s="82"/>
+      <c r="E31" s="82"/>
     </row>
     <row r="32" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
@@ -6981,11 +6982,11 @@
       <c r="B32" s="16" t="s">
         <v>562</v>
       </c>
-      <c r="C32" s="80" t="s">
+      <c r="C32" s="81" t="s">
         <v>563</v>
       </c>
-      <c r="D32" s="81"/>
-      <c r="E32" s="81"/>
+      <c r="D32" s="82"/>
+      <c r="E32" s="82"/>
     </row>
     <row r="33" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
@@ -6994,11 +6995,11 @@
       <c r="B33" s="11" t="s">
         <v>565</v>
       </c>
-      <c r="C33" s="99" t="s">
+      <c r="C33" s="101" t="s">
         <v>566</v>
       </c>
-      <c r="D33" s="81"/>
-      <c r="E33" s="81"/>
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
     </row>
     <row r="34" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
@@ -7007,11 +7008,11 @@
       <c r="B34" s="16" t="s">
         <v>568</v>
       </c>
-      <c r="C34" s="80" t="s">
+      <c r="C34" s="81" t="s">
         <v>569</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
+      <c r="D34" s="82"/>
+      <c r="E34" s="82"/>
     </row>
     <row r="35" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
@@ -7020,11 +7021,11 @@
       <c r="B35" s="11" t="s">
         <v>571</v>
       </c>
-      <c r="C35" s="99" t="s">
+      <c r="C35" s="101" t="s">
         <v>572</v>
       </c>
-      <c r="D35" s="81"/>
-      <c r="E35" s="81"/>
+      <c r="D35" s="82"/>
+      <c r="E35" s="82"/>
     </row>
     <row r="36" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
@@ -7033,25 +7034,14 @@
       <c r="B36" s="16" t="s">
         <v>574</v>
       </c>
-      <c r="C36" s="80" t="s">
+      <c r="C36" s="81" t="s">
         <v>575</v>
       </c>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
+      <c r="D36" s="82"/>
+      <c r="E36" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="C29:E29"/>
     <mergeCell ref="C35:E35"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C36:E36"/>
@@ -7068,6 +7058,17 @@
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="C33:E33"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="C29:E29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7326,78 +7327,78 @@
       <c r="A21" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="B21" s="101" t="s">
+      <c r="B21" s="100" t="s">
         <v>636</v>
       </c>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
-      <c r="E21" s="81"/>
+      <c r="C21" s="82"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="82"/>
     </row>
     <row r="22" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>637</v>
       </c>
-      <c r="B22" s="102" t="s">
+      <c r="B22" s="99" t="s">
         <v>638</v>
       </c>
-      <c r="C22" s="81"/>
-      <c r="D22" s="81"/>
-      <c r="E22" s="81"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="82"/>
+      <c r="E22" s="82"/>
     </row>
     <row r="23" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="B23" s="101" t="s">
+      <c r="B23" s="100" t="s">
         <v>640</v>
       </c>
-      <c r="C23" s="81"/>
-      <c r="D23" s="81"/>
-      <c r="E23" s="81"/>
+      <c r="C23" s="82"/>
+      <c r="D23" s="82"/>
+      <c r="E23" s="82"/>
     </row>
     <row r="24" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>641</v>
       </c>
-      <c r="B24" s="102" t="s">
+      <c r="B24" s="99" t="s">
         <v>642</v>
       </c>
-      <c r="C24" s="81"/>
-      <c r="D24" s="81"/>
-      <c r="E24" s="81"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
     </row>
     <row r="25" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="B25" s="101" t="s">
+      <c r="B25" s="100" t="s">
         <v>644</v>
       </c>
-      <c r="C25" s="81"/>
-      <c r="D25" s="81"/>
-      <c r="E25" s="81"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="82"/>
+      <c r="E25" s="82"/>
     </row>
     <row r="26" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>645</v>
       </c>
-      <c r="B26" s="102" t="s">
+      <c r="B26" s="99" t="s">
         <v>646</v>
       </c>
-      <c r="C26" s="81"/>
-      <c r="D26" s="81"/>
-      <c r="E26" s="81"/>
+      <c r="C26" s="82"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="82"/>
     </row>
     <row r="27" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="B27" s="101" t="s">
+      <c r="B27" s="100" t="s">
         <v>648</v>
       </c>
-      <c r="C27" s="81"/>
-      <c r="D27" s="81"/>
-      <c r="E27" s="81"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="82"/>
+      <c r="E27" s="82"/>
     </row>
     <row r="29" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="89" t="s">
@@ -7412,78 +7413,78 @@
       <c r="A30" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="B30" s="101" t="s">
+      <c r="B30" s="100" t="s">
         <v>651</v>
       </c>
-      <c r="C30" s="81"/>
-      <c r="D30" s="81"/>
-      <c r="E30" s="81"/>
+      <c r="C30" s="82"/>
+      <c r="D30" s="82"/>
+      <c r="E30" s="82"/>
     </row>
     <row r="31" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="B31" s="102" t="s">
+      <c r="B31" s="99" t="s">
         <v>653</v>
       </c>
-      <c r="C31" s="81"/>
-      <c r="D31" s="81"/>
-      <c r="E31" s="81"/>
+      <c r="C31" s="82"/>
+      <c r="D31" s="82"/>
+      <c r="E31" s="82"/>
     </row>
     <row r="32" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="B32" s="101" t="s">
+      <c r="B32" s="100" t="s">
         <v>655</v>
       </c>
-      <c r="C32" s="81"/>
-      <c r="D32" s="81"/>
-      <c r="E32" s="81"/>
+      <c r="C32" s="82"/>
+      <c r="D32" s="82"/>
+      <c r="E32" s="82"/>
     </row>
     <row r="33" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>656</v>
       </c>
-      <c r="B33" s="102" t="s">
+      <c r="B33" s="99" t="s">
         <v>657</v>
       </c>
-      <c r="C33" s="81"/>
-      <c r="D33" s="81"/>
-      <c r="E33" s="81"/>
+      <c r="C33" s="82"/>
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
     </row>
     <row r="34" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="B34" s="101" t="s">
+      <c r="B34" s="100" t="s">
         <v>658</v>
       </c>
-      <c r="C34" s="81"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
+      <c r="C34" s="82"/>
+      <c r="D34" s="82"/>
+      <c r="E34" s="82"/>
     </row>
     <row r="35" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="B35" s="102" t="s">
+      <c r="B35" s="99" t="s">
         <v>660</v>
       </c>
-      <c r="C35" s="81"/>
-      <c r="D35" s="81"/>
-      <c r="E35" s="81"/>
+      <c r="C35" s="82"/>
+      <c r="D35" s="82"/>
+      <c r="E35" s="82"/>
     </row>
     <row r="36" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="B36" s="101" t="s">
+      <c r="B36" s="100" t="s">
         <v>662</v>
       </c>
-      <c r="C36" s="81"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
+      <c r="C36" s="82"/>
+      <c r="D36" s="82"/>
+      <c r="E36" s="82"/>
     </row>
     <row r="38" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="87" t="s">
@@ -7498,115 +7499,103 @@
       <c r="A39" s="2" t="s">
         <v>664</v>
       </c>
-      <c r="B39" s="101" t="s">
+      <c r="B39" s="100" t="s">
         <v>665</v>
       </c>
-      <c r="C39" s="81"/>
-      <c r="D39" s="81"/>
-      <c r="E39" s="81"/>
+      <c r="C39" s="82"/>
+      <c r="D39" s="82"/>
+      <c r="E39" s="82"/>
     </row>
     <row r="40" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>666</v>
       </c>
-      <c r="B40" s="102" t="s">
+      <c r="B40" s="99" t="s">
         <v>667</v>
       </c>
-      <c r="C40" s="81"/>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
+      <c r="C40" s="82"/>
+      <c r="D40" s="82"/>
+      <c r="E40" s="82"/>
     </row>
     <row r="41" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="B41" s="101" t="s">
+      <c r="B41" s="100" t="s">
         <v>668</v>
       </c>
-      <c r="C41" s="81"/>
-      <c r="D41" s="81"/>
-      <c r="E41" s="81"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="82"/>
+      <c r="E41" s="82"/>
     </row>
     <row r="42" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>669</v>
       </c>
-      <c r="B42" s="102" t="s">
+      <c r="B42" s="99" t="s">
         <v>670</v>
       </c>
-      <c r="C42" s="81"/>
-      <c r="D42" s="81"/>
-      <c r="E42" s="81"/>
+      <c r="C42" s="82"/>
+      <c r="D42" s="82"/>
+      <c r="E42" s="82"/>
     </row>
     <row r="43" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="B43" s="101" t="s">
+      <c r="B43" s="100" t="s">
         <v>672</v>
       </c>
-      <c r="C43" s="81"/>
-      <c r="D43" s="81"/>
-      <c r="E43" s="81"/>
+      <c r="C43" s="82"/>
+      <c r="D43" s="82"/>
+      <c r="E43" s="82"/>
     </row>
     <row r="44" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>673</v>
       </c>
-      <c r="B44" s="102" t="s">
+      <c r="B44" s="99" t="s">
         <v>674</v>
       </c>
-      <c r="C44" s="81"/>
-      <c r="D44" s="81"/>
-      <c r="E44" s="81"/>
+      <c r="C44" s="82"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="82"/>
     </row>
     <row r="45" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="B45" s="101" t="s">
+      <c r="B45" s="100" t="s">
         <v>676</v>
       </c>
-      <c r="C45" s="81"/>
-      <c r="D45" s="81"/>
-      <c r="E45" s="81"/>
+      <c r="C45" s="82"/>
+      <c r="D45" s="82"/>
+      <c r="E45" s="82"/>
     </row>
     <row r="46" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>677</v>
       </c>
-      <c r="B46" s="102" t="s">
+      <c r="B46" s="99" t="s">
         <v>678</v>
       </c>
-      <c r="C46" s="81"/>
-      <c r="D46" s="81"/>
-      <c r="E46" s="81"/>
+      <c r="C46" s="82"/>
+      <c r="D46" s="82"/>
+      <c r="E46" s="82"/>
     </row>
     <row r="47" spans="1:5" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>679</v>
       </c>
-      <c r="B47" s="101" t="s">
+      <c r="B47" s="100" t="s">
         <v>680</v>
       </c>
-      <c r="C47" s="81"/>
-      <c r="D47" s="81"/>
-      <c r="E47" s="81"/>
+      <c r="C47" s="82"/>
+      <c r="D47" s="82"/>
+      <c r="E47" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B33:E33"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="B22:E22"/>
@@ -7623,6 +7612,18 @@
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="B34:E34"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B33:E33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>